<commit_message>
ME5312 (16.06.2026) konteyner nomlari tuzatildi: 25х25 0,9 (5,8) endi (Ж-1) kartasiga; xato '30х25' nomi '(Ярим овал) Пр. 30х15 ст 1,1 (Ж-1)' ga (ilgari inventarga umuman mos kelmay, yuk kartalarda ko'rinmasdi); og'irliklar Xitoy birlik vazniga qayta hisoblandi
</commit_message>
<xml_diff>
--- a/konteynerlar/xitoy_parsed/ME5312_16.06.2026.xlsx
+++ b/konteynerlar/xitoy_parsed/ME5312_16.06.2026.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Yuk" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yuk" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -450,14 +450,14 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Пр. 25х25 ст 0,9 (5,8 м) (201 марка)</t>
+          <t>Пр. 25х25 ст 0,9 (5,8 м) (201 марка) (Ж-1)</t>
         </is>
       </c>
       <c r="C2" t="n">
         <v>2532</v>
       </c>
       <c r="D2" t="n">
-        <v>9874.799999999999</v>
+        <v>9596.280000000001</v>
       </c>
     </row>
     <row r="3">
@@ -466,14 +466,14 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Пр. 30х25 ст 1,1 (6 м) (201 марка)</t>
+          <t>(Ярим овал) Пр. 30х15 ст 1,1 (6 м) (201 марка) (Ж-1)</t>
         </is>
       </c>
       <c r="C3" t="n">
         <v>3422</v>
       </c>
       <c r="D3" t="n">
-        <v>12927</v>
+        <v>12935.16</v>
       </c>
     </row>
     <row r="4">
@@ -489,7 +489,7 @@
         <v>634</v>
       </c>
       <c r="D4" t="n">
-        <v>2005.98</v>
+        <v>1895.66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>